<commit_message>
Full result AI check
</commit_message>
<xml_diff>
--- a/result/icd9_inclusion_mapping_summary.xlsx
+++ b/result/icd9_inclusion_mapping_summary.xlsx
@@ -525,17 +525,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0141</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Operations on thalamus</t>
+          <t>Operations on cornea</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
+          <t>Cornea is an eye structure, not an endocrine gland.</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific aortic category.</t>
+          <t>Vitreous is an eye structure, not an endocrine gland.</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -595,17 +595,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Operations on cornea</t>
+          <t>Operations on ureter</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
+          <t>Ureter belongs to the urinary system, not endocrine glands.</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -630,17 +630,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>0141</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Operations on ureter</t>
+          <t>Operations on thalamus</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
+          <t>Thalamus is a brain structure, not an endocrine gland.</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -675,7 +675,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
+          <t>Heart septal defect is unrelated to a retinal tear.</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -710,11 +710,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G7" t="b">
-        <v>0</v>
+          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -735,21 +735,21 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1753</t>
+          <t>1754</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
+          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
+          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -770,21 +770,21 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1754</t>
+          <t>1753</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
+          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G9" t="b">
-        <v>0</v>
+          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -805,21 +805,21 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1753</t>
+          <t>1754</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
+          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific mitral category.</t>
-        </is>
-      </c>
-      <c r="G10" t="b">
-        <v>0</v>
+          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -840,21 +840,21 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1755</t>
+          <t>1753</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Transluminal coronary atherectomy</t>
+          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
+          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -875,17 +875,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1754</t>
+          <t>1755</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
+          <t>Transluminal coronary atherectomy</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific mitral category.</t>
+          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
         </is>
       </c>
       <c r="G12" t="b">
@@ -910,21 +910,21 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1753</t>
+          <t>1754</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
+          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
+          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -945,21 +945,21 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1755</t>
+          <t>1753</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Transluminal coronary atherectomy</t>
+          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G14" t="b">
-        <v>0</v>
+          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -980,17 +980,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1754</t>
+          <t>1755</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
+          <t>Transluminal coronary atherectomy</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
+          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
         </is>
       </c>
       <c r="G15" t="b">
@@ -1015,21 +1015,21 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1753</t>
+          <t>1754</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
+          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
-        </is>
-      </c>
-      <c r="G16" t="b">
-        <v>0</v>
+          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1050,21 +1050,21 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1755</t>
+          <t>1753</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Transluminal coronary atherectomy</t>
+          <t>Percutaneous atherectomy of extracranial vessel(s)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific mitral category.</t>
-        </is>
-      </c>
-      <c r="G17" t="b">
-        <v>0</v>
+          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1085,17 +1085,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1754</t>
+          <t>1755</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Percutaneous atherectomy of intracranial vessel(s)</t>
+          <t>Transluminal coronary atherectomy</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
+          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
         </is>
       </c>
       <c r="G18" t="b">
@@ -1120,21 +1120,21 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Incision of mastoid</t>
+          <t>Other mastoidectomy</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
-        </is>
-      </c>
-      <c r="G19" t="b">
-        <v>0</v>
+          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1155,21 +1155,21 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>2041</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mastoidectomy</t>
+          <t>Simple mastoidectomy</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
-        </is>
-      </c>
-      <c r="G20" t="b">
-        <v>0</v>
+          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1190,21 +1190,21 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>854</t>
+          <t>2042</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mastectomy</t>
+          <t>Radical mastoidectomy</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
-        </is>
-      </c>
-      <c r="G21" t="b">
-        <v>0</v>
+          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1225,17 +1225,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2041</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy</t>
+          <t>Incision of mastoid</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
         </is>
       </c>
       <c r="G22" t="b">
@@ -1270,11 +1270,11 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Removal of a device does not fall under insertion categories.</t>
-        </is>
-      </c>
-      <c r="G23" t="b">
-        <v>0</v>
+          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1295,21 +1295,21 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2042</t>
+          <t>204</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy</t>
+          <t>Mastoidectomy</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Removal of a device does not fall under insertion categories.</t>
-        </is>
-      </c>
-      <c r="G24" t="b">
-        <v>0</v>
+          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1330,17 +1330,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>854</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Other mastoidectomy</t>
+          <t>Mastectomy</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A diagnostic ECG is not a central venous catheter placement.</t>
+          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
         </is>
       </c>
       <c r="G25" t="b">
@@ -1365,21 +1365,21 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Incision of mastoid</t>
+          <t>Other mastoidectomy</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Duodenostomy is a distinct procedure from loop enterostomy exteriorization.</t>
-        </is>
-      </c>
-      <c r="G26" t="b">
-        <v>0</v>
+          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1400,21 +1400,21 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>2041</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Mastoidectomy</t>
+          <t>Simple mastoidectomy</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sialoadenectomy is salivary gland removal, completely unrelated to rectum.</t>
-        </is>
-      </c>
-      <c r="G27" t="b">
-        <v>0</v>
+          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1435,21 +1435,21 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>854</t>
+          <t>2042</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mastectomy</t>
+          <t>Radical mastoidectomy</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Partial proctectomy is distinct from an abdominoperineal complete proctectomy.</t>
-        </is>
-      </c>
-      <c r="G28" t="b">
-        <v>0</v>
+          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2041</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy</t>
+          <t>Incision of mastoid</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Cystectomy is bladder removal, completely unrelated to the rectum.</t>
+          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
         </is>
       </c>
       <c r="G29" t="b">
@@ -1515,11 +1515,11 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Missing target code data cannot be mapped.</t>
-        </is>
-      </c>
-      <c r="G30" t="b">
-        <v>0</v>
+          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1540,21 +1540,21 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2042</t>
+          <t>204</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy</t>
+          <t>Mastoidectomy</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Liver operations are separate from biliary tract/hepatic duct procedures.</t>
-        </is>
-      </c>
-      <c r="G31" t="b">
-        <v>0</v>
+          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1575,17 +1575,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>854</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Other mastoidectomy</t>
+          <t>Mastectomy</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Thalamus is a brain structure, not an endocrine gland.</t>
+          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
         </is>
       </c>
       <c r="G32" t="b">
@@ -1610,21 +1610,21 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Incision of mastoid</t>
+          <t>Other mastoidectomy</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Vitreous is an eye structure, not an endocrine gland.</t>
-        </is>
-      </c>
-      <c r="G33" t="b">
-        <v>0</v>
+          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1645,21 +1645,21 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>2041</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mastoidectomy</t>
+          <t>Simple mastoidectomy</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Cornea is an eye structure, not an endocrine gland.</t>
-        </is>
-      </c>
-      <c r="G34" t="b">
-        <v>0</v>
+          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1680,21 +1680,21 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>854</t>
+          <t>2042</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mastectomy</t>
+          <t>Radical mastoidectomy</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Ureter belongs to the urinary system, not endocrine glands.</t>
-        </is>
-      </c>
-      <c r="G35" t="b">
-        <v>0</v>
+          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1715,17 +1715,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2041</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy</t>
+          <t>Incision of mastoid</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Heart septal defect is unrelated to a retinal tear.</t>
+          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
         </is>
       </c>
       <c r="G36" t="b">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
         </is>
       </c>
       <c r="G37" s="3" t="b">
@@ -1785,17 +1785,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2042</t>
+          <t>204</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy</t>
+          <t>Mastoidectomy</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
+          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
         </is>
       </c>
       <c r="G38" s="3" t="b">
@@ -1820,21 +1820,21 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>854</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Other mastoidectomy</t>
+          <t>Mastectomy</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="b">
-        <v>1</v>
+          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
+        </is>
+      </c>
+      <c r="G39" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1855,21 +1855,21 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Operations on lens</t>
+          <t>Operations on liver</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="b">
-        <v>1</v>
+          <t>Liver belongs to the digestive system, not mouth/face.</t>
+        </is>
+      </c>
+      <c r="G40" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1890,17 +1890,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Operations on eyelids</t>
+          <t>Operations on tongue</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
+          <t>Tongue operations are separate from lips under mouth codes.</t>
         </is>
       </c>
       <c r="G41" t="b">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Operations on liver</t>
+          <t>Operations on eyelids</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Suture of intestinal laceration is not a hernia repair.</t>
+          <t>Eyelids belong to the eye region, not mouth/face.</t>
         </is>
       </c>
       <c r="G42" t="b">
@@ -1960,17 +1960,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Operations on tongue</t>
+          <t>Operations on lens</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Suture of intestinal laceration is not a hernia repair.</t>
+          <t>Lens is part of the eye, not mouth/face.</t>
         </is>
       </c>
       <c r="G43" t="b">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>The anus is part of the lower GI tract, not flank.</t>
+          <t>Tongue operations are separate from palate under mouth codes.</t>
         </is>
       </c>
       <c r="G44" t="b">
@@ -2030,17 +2030,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>The lens is in the eye, unrelated to the flank.</t>
+          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G45" t="b">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>The thalamus is in the brain, unrelated to the flank.</t>
+          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G46" t="b">
@@ -2100,17 +2100,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>The vitreous is in the eye, unrelated to the flank.</t>
+          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G47" t="b">
@@ -2135,17 +2135,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>The cornea is in the eye, unrelated to the flank.</t>
+          <t>Unspecified heart valve is outside the specific aortic category.</t>
         </is>
       </c>
       <c r="G48" t="b">
@@ -2170,17 +2170,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>The ureter is part of the urinary tract, not abdominal flank.</t>
+          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G49" t="b">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>The ovary belongs to the female reproductive system, not peritoneum.</t>
+          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G50" t="b">
@@ -2240,17 +2240,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Bladder procedures are distinct from kidney and renal pelvis operations.</t>
+          <t>Unspecified heart valve is outside the specific aortic category.</t>
         </is>
       </c>
       <c r="G51" t="b">
@@ -2285,11 +2285,11 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="b">
-        <v>1</v>
+          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
+        </is>
+      </c>
+      <c r="G52" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2310,21 +2310,21 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="b">
-        <v>1</v>
+          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
+        </is>
+      </c>
+      <c r="G53" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
+          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
         </is>
       </c>
       <c r="G54" t="b">
@@ -2380,21 +2380,21 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="b">
-        <v>1</v>
+          <t>Unspecified heart valve is outside the specific aortic category.</t>
+        </is>
+      </c>
+      <c r="G55" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2425,11 +2425,11 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Extracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="b">
-        <v>1</v>
+          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
+        </is>
+      </c>
+      <c r="G56" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Coronary vessels are explicitly excluded from non-coronary categories.</t>
+          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G57" t="b">
@@ -2485,21 +2485,21 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Intracranial vessels are non-coronary, matching the parent category.</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="b">
-        <v>1</v>
+          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
+        </is>
+      </c>
+      <c r="G58" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2520,17 +2520,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
+          <t>Unspecified heart valve is outside the specific mitral category.</t>
         </is>
       </c>
       <c r="G59" t="b">
@@ -2555,21 +2555,21 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="b">
-        <v>1</v>
+          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
+        </is>
+      </c>
+      <c r="G60" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -2590,17 +2590,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
+          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G61" t="b">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Missing target code data cannot be mapped.</t>
+          <t>Unspecified heart valve is outside the specific mitral category.</t>
         </is>
       </c>
       <c r="G62" t="b">
@@ -2660,17 +2660,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Surgical removal (salpingectomy) is not a destruction/occlusion procedure.</t>
+          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G63" t="b">
@@ -2695,17 +2695,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Embolization with coils explicitly contradicts the without coils parent category.</t>
+          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G64" t="b">
@@ -2730,21 +2730,21 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Application of splint directly matches the category inclusion terms.</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="b">
-        <v>1</v>
+          <t>Pulmonary valve replacement is distinct from mitral valve replacement.</t>
+        </is>
+      </c>
+      <c r="G65" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2765,17 +2765,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>The cornea is an ocular structure, not a joint condyle.</t>
+          <t>Tricuspid valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G66" t="b">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>The thalamus is a brain structure, not a joint condyle.</t>
+          <t>Unspecified heart valve is outside the specific mitral category.</t>
         </is>
       </c>
       <c r="G67" t="b">
@@ -2835,17 +2835,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>The vitreous is an eye structure, not a joint condyle.</t>
+          <t>Aortic valve replacement is distinct from mitral valve replacement.</t>
         </is>
       </c>
       <c r="G68" t="b">
@@ -2870,17 +2870,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Missing target code data cannot be mapped.</t>
+          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
         </is>
       </c>
       <c r="G69" t="b">
@@ -2905,17 +2905,17 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Specific graft/prosthesis repairs are excluded from unspecified repair codes.</t>
+          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
         </is>
       </c>
       <c r="G70" t="b">
@@ -2940,21 +2940,21 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="b">
-        <v>1</v>
+          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
+        </is>
+      </c>
+      <c r="G71" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2975,21 +2975,21 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="b">
-        <v>1</v>
+          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
+        </is>
+      </c>
+      <c r="G72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -3010,21 +3010,21 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G73" s="3" t="b">
-        <v>1</v>
+          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
+        </is>
+      </c>
+      <c r="G73" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -3045,21 +3045,21 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="b">
-        <v>1</v>
+          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
+        </is>
+      </c>
+      <c r="G74" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -3080,21 +3080,21 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3527</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of tricuspid valve with tissue graft</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G75" s="3" t="b">
-        <v>1</v>
+          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
+        </is>
+      </c>
+      <c r="G75" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3115,21 +3115,21 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>3527</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Open and other replacement of tricuspid valve with tissue graft</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="b">
-        <v>1</v>
+          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
+        </is>
+      </c>
+      <c r="G76" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -3150,17 +3150,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Vulva operations belong to female anatomy, not male perineum.</t>
+          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
         </is>
       </c>
       <c r="G77" t="b">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>The anus is gastrointestinal, unrelated to skin nails.</t>
+          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
         </is>
       </c>
       <c r="G78" t="b">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>The lens is ocular, completely unrelated to skin nails.</t>
+          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
         </is>
       </c>
       <c r="G79" t="b">
@@ -3255,17 +3255,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Nose operations belong to respiratory/ENT, not standard skin nails.</t>
+          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
         </is>
       </c>
       <c r="G80" t="b">
@@ -3290,21 +3290,21 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Excision of skin for graft directly matches the inclusion criteria.</t>
-        </is>
-      </c>
-      <c r="G81" s="3" t="b">
-        <v>1</v>
+          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G81" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -3325,21 +3325,21 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G82" s="3" t="b">
-        <v>1</v>
+          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G82" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -3360,21 +3360,21 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G83" s="3" t="b">
-        <v>1</v>
+          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+        </is>
+      </c>
+      <c r="G83" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -3395,21 +3395,21 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G84" s="3" t="b">
-        <v>1</v>
+          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G84" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -3430,21 +3430,21 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="b">
-        <v>1</v>
+          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G85" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3465,17 +3465,17 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
+          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
         </is>
       </c>
       <c r="G86" t="b">
@@ -3500,21 +3500,21 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
-        </is>
-      </c>
-      <c r="G87" s="3" t="b">
-        <v>1</v>
+          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+        </is>
+      </c>
+      <c r="G87" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -3535,17 +3535,17 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
+          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
         </is>
       </c>
       <c r="G88" t="b">
@@ -3570,21 +3570,21 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>3525</t>
+          <t>3523</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Open and other replacement of pulmonary valve with tissue graft</t>
+          <t>Open and other replacement of mitral valve with tissue graft</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G89" s="3" t="b">
-        <v>1</v>
+          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G89" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -3605,21 +3605,21 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3521</t>
+          <t>3525</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Open and other replacement of aortic valve with tissue graft</t>
+          <t>Open and other replacement of pulmonary valve with tissue graft</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G90" s="3" t="b">
-        <v>1</v>
+          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
+        </is>
+      </c>
+      <c r="G90" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -3640,21 +3640,21 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>3523</t>
+          <t>3520</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Open and other replacement of mitral valve with tissue graft</t>
+          <t>Open and other replacement of unspecified heart valve</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G91" s="3" t="b">
-        <v>1</v>
+          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+        </is>
+      </c>
+      <c r="G91" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -3675,17 +3675,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>3520</t>
+          <t>3521</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Open and other replacement of unspecified heart valve</t>
+          <t>Open and other replacement of aortic valve with tissue graft</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
+          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
         </is>
       </c>
       <c r="G92" t="b">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
+          <t>Removal of a device does not fall under insertion categories.</t>
         </is>
       </c>
       <c r="G93" t="b">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>Removal of a device does not fall under insertion categories.</t>
         </is>
       </c>
       <c r="G94" t="b">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>A diagnostic ECG is not a central venous catheter placement.</t>
         </is>
       </c>
       <c r="G95" t="b">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>Duodenostomy is a distinct procedure from loop enterostomy exteriorization.</t>
         </is>
       </c>
       <c r="G96" t="b">
@@ -3850,17 +3850,17 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2632</t>
+          <t>576</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Complete sialoadenectomy</t>
+          <t>Partial cystectomy</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>Cystectomy is bladder removal, completely unrelated to the rectum.</t>
         </is>
       </c>
       <c r="G97" t="b">
@@ -3885,17 +3885,17 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4869</t>
+          <t>481</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Partial proctectomy</t>
+          <t>Proctostomy</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific pulmonary category.</t>
+          <t>Proctostomy is creating an opening, not a rectal resection.</t>
         </is>
       </c>
       <c r="G98" t="b">
@@ -3920,17 +3920,17 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>576</t>
+          <t>4869</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Partial cystectomy</t>
+          <t>Partial proctectomy</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>Partial proctectomy is distinct from an abdominoperineal complete proctectomy.</t>
         </is>
       </c>
       <c r="G99" t="b">
@@ -3955,12 +3955,17 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>481</t>
+          <t>2632</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Complete sialoadenectomy</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from pulmonary valve replacement.</t>
+          <t>Sialoadenectomy is salivary gland removal, completely unrelated to rectum.</t>
         </is>
       </c>
       <c r="G100" t="b">
@@ -3995,7 +4000,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>Liver operations are separate from biliary tract/hepatic duct procedures.</t>
         </is>
       </c>
       <c r="G101" t="b">
@@ -4030,11 +4035,11 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G102" s="3" t="b">
-        <v>1</v>
+          <t>Suture of intestinal laceration is not a hernia repair.</t>
+        </is>
+      </c>
+      <c r="G102" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -4065,7 +4070,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Incision is not an implantation, replacement, or mastoidectomy.</t>
+          <t>Suture of intestinal laceration is not a hernia repair.</t>
         </is>
       </c>
       <c r="G103" t="b">
@@ -4090,21 +4095,21 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Operations on anus</t>
+          <t>Operations on cornea</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Mastoidectomy matches the parent category inclusion criteria.</t>
-        </is>
-      </c>
-      <c r="G104" s="3" t="b">
-        <v>1</v>
+          <t>The cornea is in the eye, unrelated to the flank.</t>
+        </is>
+      </c>
+      <c r="G104" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -4125,17 +4130,17 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>147</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Operations on lens</t>
+          <t>Operations on vitreous</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Mastectomy is breast surgery, completely unrelated to cochlear/mastoid.</t>
+          <t>The vitreous is in the eye, unrelated to the flank.</t>
         </is>
       </c>
       <c r="G105" t="b">
@@ -4160,21 +4165,21 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>0141</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Operations on thalamus</t>
+          <t>Operations on ureter</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Simple mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G106" s="3" t="b">
-        <v>1</v>
+          <t>The ureter is part of the urinary tract, not abdominal flank.</t>
+        </is>
+      </c>
+      <c r="G106" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -4195,21 +4200,21 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>49</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Operations on vitreous</t>
+          <t>Operations on anus</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Revision of mastoidectomy falls under included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="b">
-        <v>1</v>
+          <t>The anus is part of the lower GI tract, not flank.</t>
+        </is>
+      </c>
+      <c r="G107" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -4230,21 +4235,21 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Operations on cornea</t>
+          <t>Operations on lens</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Radical mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="b">
-        <v>1</v>
+          <t>The lens is in the eye, unrelated to the flank.</t>
+        </is>
+      </c>
+      <c r="G108" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -4265,21 +4270,21 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>0141</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Operations on ureter</t>
+          <t>Operations on thalamus</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Other mastoidectomy falls under the included mastoidectomy criteria.</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="b">
-        <v>1</v>
+          <t>The thalamus is in the brain, unrelated to the flank.</t>
+        </is>
+      </c>
+      <c r="G109" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -4310,7 +4315,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Lens is part of the eye, not mouth/face.</t>
+          <t>The ovary belongs to the female reproductive system, not peritoneum.</t>
         </is>
       </c>
       <c r="G110" t="b">
@@ -4345,7 +4350,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Eyelids belong to the eye region, not mouth/face.</t>
+          <t>Bladder procedures are distinct from kidney and renal pelvis operations.</t>
         </is>
       </c>
       <c r="G111" t="b">
@@ -4373,9 +4378,14 @@
           <t>4899</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Saucerization rectum</t>
+        </is>
+      </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Arteriography visualizes arteries, whereas phlebography is strictly for veins.</t>
+          <t>The rectum belongs to the lower digestive tract, not urethra.</t>
         </is>
       </c>
       <c r="G112" t="b">
@@ -4410,7 +4420,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Angiocardiography visualizes heart chambers, not peripheral veins specifically.</t>
+          <t>Surgical removal (salpingectomy) is not a destruction/occlusion procedure.</t>
         </is>
       </c>
       <c r="G113" t="b">
@@ -4445,11 +4455,11 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Ocular ultrasound is a type of diagnostic ultrasonography.</t>
-        </is>
-      </c>
-      <c r="G114" s="3" t="b">
-        <v>1</v>
+          <t>Embolization with coils explicitly contradicts the without coils parent category.</t>
+        </is>
+      </c>
+      <c r="G114" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="115">
@@ -4480,11 +4490,11 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Non-invasive ventilation directly contradicts an invasive mechanical ventilation category.</t>
-        </is>
-      </c>
-      <c r="G115" t="b">
-        <v>0</v>
+          <t>Application of splint directly matches the category inclusion terms.</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -4515,7 +4525,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Extracorporeal circulation is a heart-lung bypass machine, not mechanical ventilation.</t>
+          <t>The cornea is an ocular structure, not a joint condyle.</t>
         </is>
       </c>
       <c r="G116" t="b">
@@ -4540,17 +4550,17 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>0141</t>
+          <t>147</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Operations on thalamus</t>
+          <t>Operations on vitreous</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Liver belongs to the digestive system, not mouth/face.</t>
+          <t>The vitreous is an eye structure, not a joint condyle.</t>
         </is>
       </c>
       <c r="G117" t="b">
@@ -4575,17 +4585,17 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>0141</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Operations on vitreous</t>
+          <t>Operations on thalamus</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Tongue operations are separate from lips under mouth codes.</t>
+          <t>The thalamus is a brain structure, not a joint condyle.</t>
         </is>
       </c>
       <c r="G118" t="b">
@@ -4613,13 +4623,18 @@
           <t>8199</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ligament NEC</t>
+        </is>
+      </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Tongue operations are separate from palate under mouth codes.</t>
-        </is>
-      </c>
-      <c r="G119" t="b">
-        <v>0</v>
+          <t>Operations on a ligament match the inclusion criteria for joints.</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -4650,7 +4665,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
+          <t>Specific graft/prosthesis repairs are excluded from unspecified repair codes.</t>
         </is>
       </c>
       <c r="G120" t="b">
@@ -4685,11 +4700,11 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
-        </is>
-      </c>
-      <c r="G121" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -4720,11 +4735,11 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific aortic category.</t>
-        </is>
-      </c>
-      <c r="G122" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -4755,11 +4770,11 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Tricuspid valve replacement is distinct from aortic valve replacement.</t>
-        </is>
-      </c>
-      <c r="G123" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -4790,11 +4805,11 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific aortic category.</t>
-        </is>
-      </c>
-      <c r="G124" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -4825,11 +4840,11 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from aortic valve replacement.</t>
-        </is>
-      </c>
-      <c r="G125" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="126">
@@ -4860,11 +4875,11 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from aortic valve replacement.</t>
-        </is>
-      </c>
-      <c r="G126" t="b">
-        <v>0</v>
+          <t>Excision/diskectomy is a necessary component of spinal prosthesis insertion.</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -4895,7 +4910,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>Vulva operations belong to female anatomy, not male perineum.</t>
         </is>
       </c>
       <c r="G127" t="b">
@@ -4930,7 +4945,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>The anus is gastrointestinal, unrelated to skin nails.</t>
         </is>
       </c>
       <c r="G128" t="b">
@@ -4955,17 +4970,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Operations on lens</t>
+          <t>Operations on nose</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+          <t>Nose operations belong to respiratory/ENT, not standard skin nails.</t>
         </is>
       </c>
       <c r="G129" t="b">
@@ -4990,17 +5005,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Operations on nose</t>
+          <t>Operations on lens</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>The lens is ocular, completely unrelated to skin nails.</t>
         </is>
       </c>
       <c r="G130" t="b">
@@ -5035,11 +5050,11 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
-        </is>
-      </c>
-      <c r="G131" t="b">
-        <v>0</v>
+          <t>Excision of skin for graft directly matches the inclusion criteria.</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -5060,17 +5075,17 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>884</t>
+          <t>885</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Arteriography using contrast material</t>
+          <t>Angiocardiography using contrast material</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>Angiocardiography visualizes heart chambers, not peripheral veins specifically.</t>
         </is>
       </c>
       <c r="G132" t="b">
@@ -5095,17 +5110,17 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>885</t>
+          <t>884</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Angiocardiography using contrast material</t>
+          <t>Arteriography using contrast material</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Unspecified heart valve is outside the specific tricuspid category.</t>
+          <t>Arteriography visualizes arteries, whereas phlebography is strictly for veins.</t>
         </is>
       </c>
       <c r="G133" t="b">
@@ -5140,11 +5155,11 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Pulmonary valve replacement is distinct from tricuspid valve replacement.</t>
-        </is>
-      </c>
-      <c r="G134" t="b">
-        <v>0</v>
+          <t>Ocular ultrasound is a type of diagnostic ultrasonography.</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -5175,7 +5190,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Aortic valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>Non-invasive ventilation directly contradicts an invasive mechanical ventilation category.</t>
         </is>
       </c>
       <c r="G135" t="b">
@@ -5210,7 +5225,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Mitral valve replacement is distinct from tricuspid valve replacement.</t>
+          <t>Extracorporeal circulation is a heart-lung bypass machine, not mechanical ventilation.</t>
         </is>
       </c>
       <c r="G136" t="b">

</xml_diff>